<commit_message>
Add new permissionset for BRLPrtyLeaseMgtPerm and update various pages and reports with captions and usage categories
</commit_message>
<xml_diff>
--- a/Unearned Rent Revenue.xlsx
+++ b/Unearned Rent Revenue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28523"/>
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28821"/>
   <x:workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\BcCore\Platform\Server\Prod.Ncl\Runtime\Office\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Depot\BcCore\Platform\Server\Prod.Ncl\Runtime\Office\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C047C7D7-11EE-4DA8-AAC2-1AF211845798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFC384A2-C507-4D37-A98A-C7420B7BE849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
-    <x:workbookView xWindow="-71110" yWindow="3060" windowWidth="28800" windowHeight="15320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <x:workbookView xWindow="0" yWindow="540" windowWidth="30825" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -19,31 +19,35 @@
     <x:sheet name="Aggregated Metadata" sheetId="4" r:id="rId4"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="ReportMetadata.AboutThisReportText" comment="Use this function to get the About This Report Text from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Text",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.AboutThisReportTitle" comment="Use this function to get the About This Report Title from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Title",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionID" comment="Use this function to get the Extension ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionName" comment="Use this function to get the Extension Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionPublisher" comment="Use this function to get the Extension Publisher from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Publisher",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ExtensionVersion" comment="Use this function to get the Extension Version from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Version",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ObjectID" comment="Use this function to get the Object ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ObjectName" comment="Use this function to get the Object Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportMetadata.ReportHelpLink" comment="Use this function to get the Report help link from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Report help link",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.CompanyId" comment="Use this function to get the Company Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.CompanyName" comment="Use this function to get the Company name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.CompanyDisplayName" comment="Use this function to get the Company display name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company display name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.Date" comment="Use this function to get the Date from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.EnvironmentName" comment="Use this function to get the Environment name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.EnvironmentType" comment="Use this function to get the Environment type from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment type",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.FormatRegion" comment="Use this function to get the Format Region from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Format Region",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.Language" comment="Use this function to get the Language from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Language",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.TenantEntraId" comment="Use this function to get the Tenant Entra Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Entra Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.LayoutName" comment="Use this function to get the Layout name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.LayoutCaption" comment="Use this function to get the Layout caption from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout caption",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
-    <x:definedName name="ReportRequest.LayoutId" comment="Use this function to get the Layout id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none",)</x:definedName>
+    <x:definedName name="ReportMetadata.AboutThisReportText" comment="Use this function to get the About This Report Text from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Text",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.AboutThisReportTitle" comment="Use this function to get the About This Report Title from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("About This Report Title",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ExtensionName" comment="Use this function to get the Extension Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ExtensionPublisher" comment="Use this function to get the Extension Publisher from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Publisher",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ExtensionVersion" comment="Use this function to get the Extension Version from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension Version",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ObjectCaption" comment="Use this function to get the Object Caption from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Caption",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ObjectID" comment="Use this function to get the Object ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ObjectName" comment="Use this function to get the Object Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Name",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ReportHelpLink" comment="Use this function to get the Report help link from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Report help link",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.CompanyDisplayName" comment="Use this function to get the Company Display name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company display name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.CompanyId" comment="Use this function to get the Company Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.CompanyName" comment="Use this function to get the Company name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.Date" comment="Use this function to get the Date from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.DateLocal" comment="Use this function to get the Date (Local) from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date (Local)",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.EnvironmentName" comment="Use this function to get the Environment name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.EnvironmentType" comment="Use this function to get the Environment type from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment type",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.FormatRegion" comment="Use this function to get the Format Region from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Format Region",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.Language" comment="Use this function to get the Language from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Language",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.LayoutCaption" comment="Use this function to get the Layout caption from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout caption",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.LayoutId" comment="Use this function to get the Layout id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.LayoutName" comment="Use this function to get the Layout name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.TenantEntraId" comment="Use this function to get the Tenant Entra Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Entra Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportRequest.UTCOffset" comment="Use this function to get the UTC Offset from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("UTC Offset",ReportRequestValues[[#All],[Request Property]],ReportRequestValues[[#All],[Request Property Value]],"none")</x:definedName>
+    <x:definedName name="ReportMetadata.ExtensionID" comment="Use this function to get the Extension Id from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Extension ID",ReportMetadataValues[[#All],[Report Property]],ReportMetadataValues[[#All],[Report Property Value]],"none")</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="191029"/>
+  <x:fileRecoveryPr repairLoad="1"/>
   <x:extLst>
     <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -61,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
   <si>
     <t>TemplateColumn</t>
   </si>
@@ -241,6 +245,24 @@
   </si>
   <si>
     <t>Layout id Value</t>
+  </si>
+  <si>
+    <t>Object Caption</t>
+  </si>
+  <si>
+    <t>Object Caption Value</t>
+  </si>
+  <si>
+    <t>Date (Local)</t>
+  </si>
+  <si>
+    <t>Date (Local) Value</t>
+  </si>
+  <si>
+    <t>UTC Offset</t>
+  </si>
+  <si>
+    <t>UTC Offset Value</t>
   </si>
 </sst>
 </file>
@@ -457,7 +479,7 @@
     <x:tableColumn id="13" name="Invoice_Raised_During_the_Year" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
     <x:tableColumn id="14" name="RevenueAllocated_DuringtheYear" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
     <x:tableColumn id="15" name="Unearned_Revenue_Balance" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
-    <x:tableColumn id="16" name="CalculatedUnearnedRevBalance" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
+    <x:tableColumn id="16" name="G_L_Balance" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
     <x:tableColumn id="17" name="Shortfall_Excess" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -488,8 +510,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}" name="ReportMetadataValues" displayName="ReportMetadataValues" ref="A1:B10" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:B10" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}" name="ReportMetadataValues" displayName="ReportMetadataValues" ref="A1:B11" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:B11" xr:uid="{134EB915-8B19-4838-BDED-CECBACACF4F9}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{5CBC1C08-5A8D-42BB-92CA-C3F1D0EF0A4D}" name="Report Property"/>
     <tableColumn id="2" xr3:uid="{920E2177-8B70-4968-B161-4C2CF0A824C6}" name="Report Property Value"/>
@@ -499,8 +521,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}" name="ReportRequestValues" displayName="ReportRequestValues" ref="D1:E15" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="D1:E15" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}" name="ReportRequestValues" displayName="ReportRequestValues" ref="D1:E17" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="D1:E17" xr:uid="{1DFF5EE2-2A86-40DE-9DFD-1E96553323F6}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E6EF2D44-8AB2-42E8-A7E3-9B148922AA59}" name="Request Property"/>
     <tableColumn id="2" xr3:uid="{FA31CE16-2D0E-4E4D-BC19-2B03E00E4B08}" name="Request Property Value"/>
@@ -829,9 +851,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{00000000-0001-0000-0000-000000000000}" mc:Ignorable="x14ac xr xr2 xr3">
   <x:dimension ref="A1:A2"/>
-  <x:sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.3828125" bestFit="1" customWidth="1"/>
+    <x:col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row>
@@ -881,7 +903,7 @@
         <x:v>Unearned_Revenue_Balance</x:v>
       </x:c>
       <x:c r="P1" t="str">
-        <x:v>CalculatedUnearnedRevBalance</x:v>
+        <x:v>G_L_Balance</x:v>
       </x:c>
       <x:c r="Q1" t="str">
         <x:v>Shortfall_Excess</x:v>
@@ -951,13 +973,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B660A3C-AF79-49CD-9630-9BBF64CB79D9}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.3828125" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -979,13 +1001,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAFD9D77-FE1A-4986-8555-546CEA41E376}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.15234375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.3828125" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -993,7 +1015,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1011,23 +1033,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63D37DBB-4AC2-46F2-B64A-5C237CE209EB}">
-  <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.69140625" customWidth="1"/>
-    <col min="2" max="2" width="40.69140625" customWidth="1"/>
-    <col min="3" max="3" width="5.69140625" customWidth="1"/>
-    <col min="4" max="4" width="25.69140625" customWidth="1"/>
-    <col min="5" max="5" width="40.69140625" customWidth="1"/>
-    <col min="6" max="6" width="5.69140625" customWidth="1"/>
-    <col min="7" max="7" width="25.69140625" customWidth="1"/>
-    <col min="8" max="8" width="40.69140625" customWidth="1"/>
-    <col min="9" max="9" width="5.69140625" customWidth="1"/>
-    <col min="10" max="10" width="40.69140625" customWidth="1"/>
-    <col min="11" max="11" width="25.69140625" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="40.7109375" customWidth="1"/>
+    <col min="6" max="6" width="5.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="8" max="8" width="40.7109375" customWidth="1"/>
+    <col min="9" max="9" width="5.7109375" customWidth="1"/>
+    <col min="10" max="10" width="40.7109375" customWidth="1"/>
+    <col min="11" max="11" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1053,7 +1075,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1079,7 +1101,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1093,7 +1115,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1107,7 +1129,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1121,7 +1143,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1135,7 +1157,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1149,12 +1171,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
         <v>38</v>
@@ -1163,12 +1185,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
         <v>40</v>
@@ -1177,12 +1199,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
         <v>42</v>
@@ -1191,43 +1213,65 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
       <c r="D11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
         <v>1</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="D12" t="s">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
         <v>45</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E14" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="D13" t="s">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="D14" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
         <v>56</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="D15" t="s">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
         <v>58</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E17" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>